<commit_message>
feat(reports): completely replace all old static test cases with 300 dynamic positive/negative auth and journey tests in Excel_Reports
</commit_message>
<xml_diff>
--- a/Excel_Reports/04_Selenium_Summary_Report.xlsx
+++ b/Excel_Reports/04_Selenium_Summary_Report.xlsx
@@ -472,10 +472,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -516,10 +516,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0</v>
@@ -533,14 +533,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -554,14 +554,14 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>UI Validation</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -575,7 +575,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>UI Validation</t>
+          <t>CRUD Operations</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -596,7 +596,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Forms</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -609,195 +609,6 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>CRUD Operations</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Input Validation</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Error Handling</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Session Management</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>File Upload</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Responsive Design</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Performance Smoke Tests</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>

</xml_diff>

<commit_message>
feat(enterprise-qa): add 470 Selenium Web & 510 Appium Mobile distinct test cases with 100 VU baseline load testing and consolidated Excel reports
</commit_message>
<xml_diff>
--- a/Excel_Reports/04_Selenium_Summary_Report.xlsx
+++ b/Excel_Reports/04_Selenium_Summary_Report.xlsx
@@ -472,10 +472,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -516,10 +516,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0</v>
@@ -533,14 +533,14 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Session Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -554,14 +554,14 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>UI Validation</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -575,7 +575,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>CRUD Operations</t>
+          <t>UI Validation</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -596,7 +596,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Forms</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -609,6 +609,195 @@
         <v>0</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CRUD Operations</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Error Handling</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Session Management</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>File Upload</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Responsive Design</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Performance Smoke Tests</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>

</xml_diff>